<commit_message>
Add requirements file and update constraints workbook
</commit_message>
<xml_diff>
--- a/constraints.xlsx
+++ b/constraints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bobbyboyd/peer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C6F4F7-3F21-7049-B657-BC8AA6143041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE48E90-1DD7-D04A-9A13-1F294F277680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15020" yWindow="4500" windowWidth="19180" windowHeight="17180" activeTab="1" xr2:uid="{F8885288-F350-8444-8C3C-20F550782FD8}"/>
   </bookViews>
@@ -167,9 +167,6 @@
     <t>8 Gy</t>
   </si>
   <si>
-    <t>12 Gy</t>
-  </si>
-  <si>
     <t>23 Gy</t>
   </si>
   <si>
@@ -180,6 +177,9 @@
   </si>
   <si>
     <t>Chiasm</t>
+  </si>
+  <si>
+    <t>12-15 Gy</t>
   </si>
 </sst>
 </file>
@@ -1680,7 +1680,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
         <v>44</v>
@@ -1692,12 +1692,12 @@
         <v>6</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -1709,7 +1709,7 @@
         <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -1718,7 +1718,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1744,7 +1744,7 @@
         <v>6</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1775,7 +1775,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
         <v>5</v>
@@ -1784,7 +1784,7 @@
         <v>6</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>